<commit_message>
Actualizacion completa del sistema de convalidaciones
</commit_message>
<xml_diff>
--- a/Carreras/Ingeniería de sistemas e IA/alumnos.xlsx
+++ b/Carreras/Ingeniería de sistemas e IA/alumnos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ENRIQUE\Desktop\SISTEMA_CONVALIDACIONES\Carreras\Ingeniería de sistemas e IA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E018201-B66C-4837-A7F5-30C11F2203F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F819B637-9A6B-43CA-B8AB-42BBEFE8809C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -503,7 +503,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -516,6 +516,25 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -568,12 +587,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1257,16 +1279,16 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="5">
         <v>46201175</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="5">
         <v>942479595</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="5" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1355,16 +1377,16 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+      <c r="A33" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="5">
         <v>42804497</v>
       </c>
-      <c r="C33" s="1">
+      <c r="C33" s="5">
         <v>948462828</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="5" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1439,16 +1461,16 @@
       </c>
     </row>
     <row r="39" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
+      <c r="A39" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="3">
         <v>75582408</v>
       </c>
-      <c r="C39" s="1">
+      <c r="C39" s="3">
         <v>969601807</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="3" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1551,16 +1573,16 @@
       </c>
     </row>
     <row r="47" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
+      <c r="A47" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C47" s="1">
+      <c r="C47" s="4">
         <v>928459489</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D47" s="4" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1607,16 +1629,16 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
+      <c r="A51" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B51" s="4">
         <v>70282038</v>
       </c>
-      <c r="C51" s="1">
+      <c r="C51" s="4">
         <v>910683462</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D51" s="4" t="s">
         <v>102</v>
       </c>
     </row>

</xml_diff>